<commit_message>
Commit on 12th August
</commit_message>
<xml_diff>
--- a/Auto-IT/Bulk-Employee-Stable.xlsx
+++ b/Auto-IT/Bulk-Employee-Stable.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{274E3CDC-4E03-44F8-9CD8-8B22DF5C2582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{B5004847-4A40-4CBD-97E5-BB7F495EFE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19460" windowHeight="11060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="19460" windowHeight="11060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1282,9 +1282,6 @@
     <t>Management</t>
   </si>
   <si>
-    <t>bulkemployeeone@gmail.com</t>
-  </si>
-  <si>
     <t>Dela Supervisor One</t>
   </si>
   <si>
@@ -1303,7 +1300,10 @@
     <t>2029-01-09</t>
   </si>
   <si>
-    <t>BulkEmployeeOne</t>
+    <t>BulkEmployeeTwo</t>
+  </si>
+  <si>
+    <t>bulkemployeetwo@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1940,7 +1940,7 @@
     </row>
     <row r="2" spans="1:66" ht="15.75" customHeight="1">
       <c r="A2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>69</v>
@@ -1951,17 +1951,17 @@
       <c r="D2" s="13">
         <v>9128327231</v>
       </c>
-      <c r="E2" s="11" t="s">
-        <v>198</v>
+      <c r="E2" s="16" t="s">
+        <v>205</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>196</v>
       </c>
       <c r="G2" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H2" s="14" t="s">
         <v>203</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>204</v>
       </c>
       <c r="I2" s="13">
         <v>9238372837341</v>
@@ -2099,7 +2099,7 @@
         <v>87</v>
       </c>
       <c r="BB2" s="15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="BC2" s="6" t="s">
         <v>89</v>
@@ -2111,7 +2111,7 @@
         <v>90</v>
       </c>
       <c r="BF2" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="BG2" s="17" t="s">
         <v>109</v>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="BI2" s="18"/>
       <c r="BJ2" s="19" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="BK2" s="15">
         <v>5</v>
@@ -2133,7 +2133,7 @@
         <v>1</v>
       </c>
       <c r="BN2" s="20" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:66" ht="15.75" customHeight="1">

</xml_diff>